<commit_message>
Flag suspicious TRENCH CUT instead of hiding it
- Provenance tracking: rows summed for TRENCH CUT are recorded as
  '<sheet> row N'; shown in a red bold '!! CHECK' note in the Summary
  and on the console when the figures are inconsistent
- Sanity check triggers when TRENCH CUT exceeds TOTAL SITE CUT on any
  volume (i.e. SITE CUT ONLY would go negative - double counting in the
  export, as seen on the Bulla Road file)
- Fixture now reproduces the trap structures (hidden duplicates, per-run
  groups); negative-path test asserts the warning fires

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dev_tests/fixture_result.xlsx
+++ b/dev_tests/fixture_result.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,26 +549,42 @@
         <v>458.608016833591</v>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" t="n">
+    <row r="11" hidden="1" outlineLevel="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>All Stormwater Drainage in Trenching site</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>458.608016833591</v>
+      </c>
+      <c r="G11" t="n">
+        <v>458.608016833591</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-29.9306489</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
         <v>1674.681</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C13" t="n">
         <v>1505.325</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>3180.007</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E13" t="n">
         <v>1505.325</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F13" t="n">
         <v>3638.963</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G13" t="n">
         <v>5144.288</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H13" t="n">
         <v>1964.281</v>
       </c>
     </row>
@@ -953,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1033,42 +1049,80 @@
         <v>-258.22757067882</v>
       </c>
     </row>
-    <row r="4" hidden="1">
+    <row r="4" hidden="1" outlineLevel="1">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Cut - Trench Run 1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>129.11</v>
+      </c>
+      <c r="C4" t="n">
+        <v>116.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>245.21</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-129.11</v>
+      </c>
+    </row>
+    <row r="5" hidden="1" outlineLevel="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cut - Trench Run 2</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>129.12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>116.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>245.22</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-129.12</v>
+      </c>
+    </row>
+    <row r="6" hidden="1" outlineLevel="1">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>TrenchNetwork : Stormwater Drainage</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F6" t="n">
         <v>458.608016833591</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G6" t="n">
         <v>458.608016833591</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H6" t="n">
         <v>458.608016833591</v>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" t="n">
+    <row r="7">
+      <c r="B7" t="n">
         <v>0</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F7" t="n">
         <v>458.608</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G7" t="n">
         <v>458.608</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H7" t="n">
         <v>458.608</v>
       </c>
     </row>
@@ -1558,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1619,58 +1673,90 @@
         <v>350.302661775843</v>
       </c>
     </row>
-    <row r="4">
+    <row r="3" hidden="1" outlineLevel="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>375MM RCP PIPES - TRENCH RUN 1 - UNDER STRUCTURE</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>7.095730179</v>
+      </c>
+      <c r="G3" t="n">
+        <v>7.095730179</v>
+      </c>
+      <c r="H3" t="n">
+        <v>7.095730179</v>
+      </c>
+    </row>
+    <row r="4" hidden="1" outlineLevel="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Class 3</t>
+          <t>300MM RCP PIPES - TRENCH RUN 14 - UNDER STRUCTURE</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>69.00682717402771</v>
+        <v>0.682576877</v>
       </c>
       <c r="G4" t="n">
-        <v>69.00682717402771</v>
+        <v>0.682576877</v>
       </c>
       <c r="H4" t="n">
-        <v>69.00682717402771</v>
+        <v>0.682576877</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Class 3</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>69.00682717402771</v>
+      </c>
+      <c r="G6" t="n">
+        <v>69.00682717402771</v>
+      </c>
+      <c r="H6" t="n">
+        <v>69.00682717402771</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Site Dirt</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F8" t="n">
         <v>39.2985278837208</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G8" t="n">
         <v>39.2985278837208</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H8" t="n">
         <v>39.2985278837208</v>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" t="n">
+    <row r="10">
+      <c r="B10" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F10" t="n">
         <v>458.608</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G10" t="n">
         <v>458.608</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H10" t="n">
         <v>458.608</v>
       </c>
     </row>
@@ -1789,7 +1875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1809,89 +1895,110 @@
     <row r="3" hidden="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 300mm RCP Pipes (19 items) Quantity Total length : 405.433m</t>
+          <t>TrenchRun : Trench Run 1 (1 item) Quantity Total length : 32.305m</t>
         </is>
       </c>
     </row>
     <row r="4" hidden="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 375mm RCP Pipes (1 item) Quantity Total length : 12.091m</t>
+          <t>TrenchSegment</t>
         </is>
       </c>
     </row>
     <row r="5" hidden="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 450mm RCP Pipe (2 items) Quantity Total length : 32.373m</t>
+          <t>A - B</t>
         </is>
       </c>
     </row>
     <row r="6" hidden="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 600mm RCP Pipe (3 items) Quantity Total length : 52.048m</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>TrenchNetwork : 300mm RCP Pipes (19 items) Quantity Total length : 405.433m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" hidden="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Category : Stormwater Pit (8 items) Quantity Total length : 23.135m</t>
+          <t>TrenchNetwork : 375mm RCP Pipes (1 item) Quantity Total length : 12.091m</t>
         </is>
       </c>
     </row>
     <row r="8" hidden="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 1200 x 1200mm Grated Side Entry Pit (2 items) Quantity Total length : 2.698m</t>
+          <t>TrenchNetwork : 450mm RCP Pipe (2 items) Quantity Total length : 32.373m</t>
         </is>
       </c>
     </row>
     <row r="9" hidden="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 1500 x 1500mm Grated Entry Side Pit (1 item) Quantity Total length : 1.651m</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" hidden="1">
+          <t>TrenchNetwork : 600mm RCP Pipe (3 items) Quantity Total length : 52.048m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 1875 x 1800mm Grated Side Entry Pit Fitted with Altan Flow Filter (1 item) Quantity Total length : 2.265m</t>
+          <t>Category : Stormwater Pit (8 items) Quantity Total length : 23.135m</t>
         </is>
       </c>
     </row>
     <row r="11" hidden="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 900 x 600mm Grated Side Entry Pit (1 item) Quantity Total length : 0.753m</t>
+          <t>TrenchNetwork : 1200 x 1200mm Grated Side Entry Pit (2 items) Quantity Total length : 2.698m</t>
         </is>
       </c>
     </row>
     <row r="12" hidden="1">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 900 x 900mm Grated Inlet Pit (4 items) Quantity Total length : 4.207m</t>
+          <t>TrenchNetwork : 1500 x 1500mm Grated Entry Side Pit (1 item) Quantity Total length : 1.651m</t>
         </is>
       </c>
     </row>
     <row r="13" hidden="1">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 900 x 900mm Grated Side Entry Pit (5 items) Quantity Total length : 5.260m</t>
+          <t>TrenchNetwork : 1875 x 1800mm Grated Side Entry Pit Fitted with Altan Flow Filter (1 item) Quantity Total length : 2.265m</t>
         </is>
       </c>
     </row>
     <row r="14" hidden="1">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TrenchNetwork : 900 x 900mm Junction Pit (3 items) Quantity Total length : 3.153m</t>
+          <t>TrenchNetwork : 900 x 600mm Grated Side Entry Pit (1 item) Quantity Total length : 0.753m</t>
         </is>
       </c>
     </row>
     <row r="15" hidden="1">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>TrenchNetwork : 900 x 900mm Grated Inlet Pit (4 items) Quantity Total length : 4.207m</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TrenchNetwork : 900 x 900mm Grated Side Entry Pit (5 items) Quantity Total length : 5.260m</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" hidden="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TrenchNetwork : 900 x 900mm Junction Pit (3 items) Quantity Total length : 3.153m</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" hidden="1">
+      <c r="A18" t="inlineStr">
         <is>
           <t>TrenchNetwork : 900 x 900mm Side Entry Pit (3 items) Quantity Total length : 3.148m</t>
         </is>

</xml_diff>